<commit_message>
Add status sheet to accountant expense report
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DVpXqei8SkhtudMXpKxe2v
</commit_message>
<xml_diff>
--- a/invoices/exports/expenses-2026-05-06.xlsx
+++ b/invoices/exports/expenses-2026-05-06.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הוצאות מאי-יוני 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="סטטוס" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="הוצאות מאי-יוני 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +42,18 @@
     <font>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F7A33"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B45F06"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -78,6 +91,9 @@
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,6 +459,167 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>סטטוס מערכת איסוף החשבוניות — נכון ל-13.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>רכיב</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>מצב</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>איסוף מהמייל (osherv55@gmail.com), מאי-יוני 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>הושלם — 285 מסמכים בטבלה המרכזית</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>דוח הוצאות לרו"ח (גיליון "הוצאות מאי-יוני 2026")</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>מוכן — 236 מסמכי הוצאה, 217 עם סכום מלא</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>סה"כ הוצאות בש"ח (כולל המרות מט"ח לפי שער יומי)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>117,641.95 ₪</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>הכנסות שזוהו (לא בדוח זה)</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>39,550 ₪ — קורס + מסוף אשראי</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>סנכרון יומי אוטומטי מייל→דרייב (6:00)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>פעיל</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>בדיקה והשלמה אוטומטית שלי (4 פעמים ביום)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>פעילה</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>בהשלמה אוטומטית בימים הקרובים</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>4 קבלות מתחילת מאי (פתאל, סופר-פארם, אייס, קייטנה)</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>ממתין לריצת הסנכרון הבאה</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>14 חיובי רבו פילאטיס (הוצאה אישית, כנראה לא רלוונטי לרו"ח)</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>דורש הרצת גרסה 4 של הסקריפט</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>חשבונית צמרת מימונים</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>זמינה רק בהתחברות לאתר שלהם — ידני</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -528,7 +705,6 @@
       <c r="G2" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,7 +736,6 @@
       <c r="G3" s="2" t="n">
         <v>155.93</v>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -592,7 +767,6 @@
       <c r="G4" s="2" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -624,7 +798,6 @@
       <c r="G5" s="2" t="n">
         <v>268.9</v>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -656,7 +829,6 @@
       <c r="G6" s="2" t="n">
         <v>93.18000000000001</v>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -688,7 +860,6 @@
       <c r="G7" s="2" t="n">
         <v>201.2</v>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -720,7 +891,6 @@
       <c r="G8" s="2" t="n">
         <v>25.9</v>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -752,7 +922,6 @@
       <c r="G9" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -892,7 +1061,6 @@
       <c r="G13" s="2" t="n">
         <v>57.25</v>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -924,7 +1092,6 @@
       <c r="G14" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -956,7 +1123,6 @@
       <c r="G15" s="2" t="n">
         <v>137.6</v>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -988,7 +1154,6 @@
       <c r="G16" s="2" t="n">
         <v>134.3</v>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1020,7 +1185,6 @@
       <c r="G17" s="2" t="n">
         <v>128.35</v>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1088,7 +1252,6 @@
       <c r="G19" s="2" t="n">
         <v>135.6</v>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1156,7 +1319,6 @@
       <c r="G21" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1188,7 +1350,6 @@
       <c r="G22" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1220,7 +1381,6 @@
       <c r="G23" s="2" t="n">
         <v>18.2</v>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1252,7 +1412,6 @@
       <c r="G24" s="2" t="n">
         <v>332.9</v>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1284,7 +1443,6 @@
       <c r="G25" s="2" t="n">
         <v>200.88</v>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1388,7 +1546,6 @@
       <c r="G28" s="2" t="n">
         <v>119.45</v>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1420,7 +1577,6 @@
       <c r="G29" s="2" t="n">
         <v>14.7</v>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1452,7 +1608,6 @@
       <c r="G30" s="2" t="n">
         <v>79.90000000000001</v>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1484,7 +1639,6 @@
       <c r="G31" s="2" t="n">
         <v>427.9</v>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1516,7 +1670,6 @@
       <c r="G32" s="2" t="n">
         <v>63.91</v>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1548,7 +1701,6 @@
       <c r="G33" s="2" t="n">
         <v>493.9</v>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1580,7 +1732,6 @@
       <c r="G34" s="2" t="n">
         <v>171.9</v>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1612,7 +1763,6 @@
       <c r="G35" s="2" t="n">
         <v>29.25</v>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1644,7 +1794,6 @@
       <c r="G36" s="2" t="n">
         <v>19.5</v>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1676,7 +1825,6 @@
       <c r="G37" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1708,7 +1856,6 @@
       <c r="G38" s="2" t="n">
         <v>480</v>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1740,7 +1887,6 @@
       <c r="G39" s="2" t="n">
         <v>214.9</v>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1772,7 +1918,6 @@
       <c r="G40" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1804,7 +1949,6 @@
       <c r="G41" s="2" t="n">
         <v>88.2</v>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1836,7 +1980,6 @@
       <c r="G42" s="2" t="n">
         <v>333.9</v>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1868,7 +2011,6 @@
       <c r="G43" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1900,7 +2042,6 @@
       <c r="G44" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1932,7 +2073,6 @@
       <c r="G45" s="2" t="n">
         <v>19.5</v>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1964,7 +2104,6 @@
       <c r="G46" s="2" t="n">
         <v>58.16</v>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1996,7 +2135,6 @@
       <c r="G47" s="2" t="n">
         <v>13.9</v>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2028,7 +2166,6 @@
       <c r="G48" s="2" t="n">
         <v>199.9</v>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2060,7 +2197,6 @@
       <c r="G49" s="2" t="n">
         <v>318.94</v>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2092,7 +2228,6 @@
       <c r="G50" s="2" t="n">
         <v>130.74</v>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2124,7 +2259,6 @@
       <c r="G51" s="2" t="n">
         <v>636.9</v>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2156,7 +2290,6 @@
       <c r="G52" s="2" t="n">
         <v>25.05</v>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2188,7 +2321,6 @@
       <c r="G53" s="2" t="n">
         <v>65.90000000000001</v>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2220,7 +2352,6 @@
       <c r="G54" s="2" t="n">
         <v>24.4</v>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2252,7 +2383,6 @@
       <c r="G55" s="2" t="n">
         <v>223.9</v>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2320,7 +2450,6 @@
       <c r="G57" s="2" t="n">
         <v>963.9</v>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2352,7 +2481,6 @@
       <c r="G58" s="2" t="n">
         <v>7.35</v>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2384,7 +2512,6 @@
       <c r="G59" s="2" t="n">
         <v>601.9</v>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2416,7 +2543,6 @@
       <c r="G60" s="2" t="n">
         <v>155.5</v>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2448,7 +2574,6 @@
       <c r="G61" s="2" t="n">
         <v>39.9</v>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2480,7 +2605,6 @@
       <c r="G62" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2512,7 +2636,6 @@
       <c r="G63" s="2" t="n">
         <v>832.6</v>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2616,7 +2739,6 @@
       <c r="G66" s="2" t="n">
         <v>21.9</v>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2648,7 +2770,6 @@
       <c r="G67" s="2" t="n">
         <v>122.4</v>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2680,7 +2801,6 @@
       <c r="G68" s="2" t="n">
         <v>227.9</v>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2712,7 +2832,6 @@
       <c r="G69" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2744,7 +2863,6 @@
       <c r="G70" s="2" t="n">
         <v>13.9</v>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2776,7 +2894,6 @@
       <c r="G71" s="2" t="n">
         <v>54.88</v>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2808,7 +2925,6 @@
       <c r="G72" s="2" t="n">
         <v>22.74</v>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2840,7 +2956,6 @@
       <c r="G73" s="2" t="n">
         <v>198.9</v>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2872,7 +2987,6 @@
       <c r="G74" s="2" t="n">
         <v>475.4</v>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2904,7 +3018,6 @@
       <c r="G75" s="2" t="n">
         <v>45.83</v>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2936,7 +3049,6 @@
       <c r="G76" s="2" t="n">
         <v>190.4</v>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2968,7 +3080,6 @@
       <c r="G77" s="2" t="n">
         <v>276.6</v>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3000,7 +3111,6 @@
       <c r="G78" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3032,7 +3142,6 @@
       <c r="G79" s="2" t="n">
         <v>19.5</v>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3064,7 +3173,6 @@
       <c r="G80" s="2" t="n">
         <v>229.6</v>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3132,7 +3240,6 @@
       <c r="G82" s="2" t="n">
         <v>213.8</v>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3164,7 +3271,6 @@
       <c r="G83" s="2" t="n">
         <v>453.9</v>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3196,7 +3302,6 @@
       <c r="G84" s="2" t="n">
         <v>116.9</v>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3228,7 +3333,6 @@
       <c r="G85" s="2" t="n">
         <v>157.9</v>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3260,7 +3364,6 @@
       <c r="G86" s="2" t="n">
         <v>304.2</v>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3364,7 +3467,6 @@
       <c r="G89" s="2" t="n">
         <v>188.9</v>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3396,7 +3498,6 @@
       <c r="G90" s="2" t="n">
         <v>37.25</v>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3428,7 +3529,6 @@
       <c r="G91" s="2" t="n">
         <v>25.9</v>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3460,7 +3560,6 @@
       <c r="G92" s="2" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3492,7 +3591,6 @@
       <c r="G93" s="2" t="n">
         <v>24.7</v>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3524,7 +3622,6 @@
       <c r="G94" s="2" t="n">
         <v>70.17</v>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3628,7 +3725,6 @@
       <c r="G97" s="2" t="n">
         <v>154.9</v>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3660,7 +3756,6 @@
       <c r="G98" s="2" t="n">
         <v>356.5</v>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3692,7 +3787,6 @@
       <c r="G99" s="2" t="n">
         <v>131.5</v>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3760,7 +3854,6 @@
       <c r="G101" s="2" t="n">
         <v>536.9</v>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3792,7 +3885,6 @@
       <c r="G102" s="2" t="n">
         <v>52.1</v>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3824,7 +3916,6 @@
       <c r="G103" s="2" t="n">
         <v>285.4</v>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4000,7 +4091,6 @@
       <c r="G108" s="2" t="n">
         <v>521.7</v>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4248,7 +4338,6 @@
       <c r="G115" s="2" t="n">
         <v>25.9</v>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4280,7 +4369,6 @@
       <c r="G116" s="2" t="n">
         <v>34.7</v>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4312,7 +4400,6 @@
       <c r="G117" s="2" t="n">
         <v>170.3</v>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4344,7 +4431,6 @@
       <c r="G118" s="2" t="n">
         <v>52.29</v>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4376,7 +4462,6 @@
       <c r="G119" s="2" t="n">
         <v>328.9</v>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4444,7 +4529,6 @@
       <c r="G121" s="2" t="n">
         <v>58.23</v>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4476,7 +4560,6 @@
       <c r="G122" s="2" t="n">
         <v>58.23</v>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4508,7 +4591,6 @@
       <c r="G123" s="2" t="n">
         <v>376.32</v>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4540,7 +4622,6 @@
       <c r="G124" s="2" t="n">
         <v>122.15</v>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4572,7 +4653,6 @@
       <c r="G125" s="2" t="n">
         <v>91.73999999999999</v>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4604,7 +4684,6 @@
       <c r="G126" s="2" t="n">
         <v>28.4</v>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4636,7 +4715,6 @@
       <c r="G127" s="2" t="n">
         <v>453.9</v>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4704,7 +4782,6 @@
       <c r="G129" s="2" t="n">
         <v>153.6</v>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4736,7 +4813,6 @@
       <c r="G130" s="2" t="n">
         <v>158.32</v>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4768,7 +4844,6 @@
       <c r="G131" s="2" t="n">
         <v>64.17</v>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4800,7 +4875,6 @@
       <c r="G132" s="2" t="n">
         <v>236.35</v>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4832,7 +4906,6 @@
       <c r="G133" s="2" t="n">
         <v>86.45</v>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4900,7 +4973,6 @@
       <c r="G135" s="2" t="n">
         <v>337.5</v>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4932,7 +5004,6 @@
       <c r="G136" s="2" t="n">
         <v>134.03</v>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4964,7 +5035,6 @@
       <c r="G137" s="2" t="n">
         <v>74.45999999999999</v>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4996,7 +5066,6 @@
       <c r="G138" s="2" t="n">
         <v>20.64</v>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5028,7 +5097,6 @@
       <c r="G139" s="2" t="n">
         <v>13.9</v>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5060,7 +5128,6 @@
       <c r="G140" s="2" t="n">
         <v>14.7</v>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5092,7 +5159,6 @@
       <c r="G141" s="2" t="n">
         <v>10.2</v>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5124,7 +5190,6 @@
       <c r="G142" s="2" t="n">
         <v>12.5</v>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5156,7 +5221,6 @@
       <c r="G143" s="2" t="n">
         <v>172</v>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5260,7 +5324,6 @@
       <c r="G146" s="2" t="n">
         <v>121</v>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5292,7 +5355,6 @@
       <c r="G147" s="2" t="n">
         <v>20.9</v>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5324,7 +5386,6 @@
       <c r="G148" s="2" t="n">
         <v>223.9</v>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5356,7 +5417,6 @@
       <c r="G149" s="2" t="n">
         <v>203.9</v>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5388,7 +5448,6 @@
       <c r="G150" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5420,7 +5479,6 @@
       <c r="G151" s="2" t="n">
         <v>436.91</v>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5452,7 +5510,6 @@
       <c r="G152" s="2" t="n">
         <v>129.9</v>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5484,7 +5541,6 @@
       <c r="G153" s="2" t="n">
         <v>35.05</v>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5516,7 +5572,6 @@
       <c r="G154" s="2" t="n">
         <v>7.9</v>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5548,7 +5603,6 @@
       <c r="G155" s="2" t="n">
         <v>473.9</v>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5580,7 +5634,6 @@
       <c r="G156" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5612,7 +5665,6 @@
       <c r="G157" s="2" t="n">
         <v>13.9</v>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5644,7 +5696,6 @@
       <c r="G158" s="2" t="n">
         <v>29.26</v>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5676,7 +5727,6 @@
       <c r="G159" s="2" t="n">
         <v>131.71</v>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5708,7 +5758,6 @@
       <c r="G160" s="2" t="n">
         <v>84.03</v>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5884,7 +5933,6 @@
       <c r="G165" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5916,7 +5964,6 @@
       <c r="G166" s="2" t="n">
         <v>145.89</v>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5948,7 +5995,6 @@
       <c r="G167" s="2" t="n">
         <v>7.35</v>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5980,7 +6026,6 @@
       <c r="G168" s="2" t="n">
         <v>25.9</v>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6048,7 +6093,6 @@
       <c r="G170" s="2" t="n">
         <v>189.5</v>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6080,7 +6124,6 @@
       <c r="G171" s="2" t="n">
         <v>39.9</v>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6148,7 +6191,6 @@
       <c r="G173" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6180,7 +6222,6 @@
       <c r="G174" s="2" t="n">
         <v>11.5</v>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -6284,7 +6325,6 @@
       <c r="G177" s="2" t="n">
         <v>21.9</v>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6316,7 +6356,6 @@
       <c r="G178" s="2" t="n">
         <v>176.8</v>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6348,7 +6387,6 @@
       <c r="G179" s="2" t="n">
         <v>165.44</v>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6380,7 +6418,6 @@
       <c r="G180" s="2" t="n">
         <v>397.9</v>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6412,7 +6449,6 @@
       <c r="G181" s="2" t="n">
         <v>75.15000000000001</v>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6444,7 +6480,6 @@
       <c r="G182" s="2" t="n">
         <v>9.9</v>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6476,7 +6511,6 @@
       <c r="G183" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6508,7 +6542,6 @@
       <c r="G184" s="2" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6540,7 +6573,6 @@
       <c r="G185" s="2" t="n">
         <v>151.9</v>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6572,7 +6604,6 @@
       <c r="G186" s="2" t="n">
         <v>83.5</v>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6604,7 +6635,6 @@
       <c r="G187" s="2" t="n">
         <v>187.9</v>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6636,7 +6666,6 @@
       <c r="G188" s="2" t="n">
         <v>67.41</v>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6668,7 +6697,6 @@
       <c r="G189" s="2" t="n">
         <v>111.7</v>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6700,7 +6728,6 @@
       <c r="G190" s="2" t="n">
         <v>155.9</v>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6732,7 +6759,6 @@
       <c r="G191" s="2" t="n">
         <v>242.3</v>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6764,7 +6790,6 @@
       <c r="G192" s="2" t="n">
         <v>147.1</v>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6796,7 +6821,6 @@
       <c r="G193" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6828,7 +6852,6 @@
       <c r="G194" s="2" t="n">
         <v>5.9</v>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6860,7 +6883,6 @@
       <c r="G195" s="2" t="n">
         <v>101.05</v>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6928,7 +6950,6 @@
       <c r="G197" s="2" t="n">
         <v>204.7</v>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -6960,7 +6981,6 @@
       <c r="G198" s="2" t="n">
         <v>88.98</v>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6992,7 +7012,6 @@
       <c r="G199" s="2" t="n">
         <v>215.3</v>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -7024,7 +7043,6 @@
       <c r="G200" s="2" t="n">
         <v>99.58</v>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -7056,7 +7074,6 @@
       <c r="G201" s="2" t="n">
         <v>102.1</v>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -7088,7 +7105,6 @@
       <c r="G202" s="2" t="n">
         <v>59.96</v>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -7120,7 +7136,6 @@
       <c r="G203" s="2" t="n">
         <v>348.71</v>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -7152,7 +7167,6 @@
       <c r="G204" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7184,7 +7198,6 @@
       <c r="G205" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7216,7 +7229,6 @@
       <c r="G206" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -7248,7 +7260,6 @@
       <c r="G207" s="2" t="n">
         <v>41.3</v>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -7280,7 +7291,6 @@
       <c r="G208" s="2" t="n">
         <v>453.9</v>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -7348,7 +7358,6 @@
       <c r="G210" s="2" t="n">
         <v>519.6</v>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -7416,7 +7425,6 @@
       <c r="G212" s="2" t="n">
         <v>161.9</v>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -7448,7 +7456,6 @@
       <c r="G213" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -7480,7 +7487,6 @@
       <c r="G214" s="2" t="n">
         <v>186.9</v>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">

</xml_diff>